<commit_message>
fix: preserve letter-suffixed equipment identities (4.2.1)
</commit_message>
<xml_diff>
--- a/tests/fixtures/compiler-chain-mel.xlsx
+++ b/tests/fixtures/compiler-chain-mel.xlsx
@@ -409,7 +409,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H8"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -439,10 +439,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="str">
-        <v>GIS-01-A</v>
+        <v>GIS-01</v>
       </c>
       <c r="B2" s="2" t="str">
-        <v>Gas insulated switchgear side A</v>
+        <v>Gas insulated switchgear</v>
       </c>
       <c r="C2" s="2" t="str">
         <v>B14</v>
@@ -465,10 +465,10 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="str">
-        <v>GIS-01-B</v>
+        <v>GIS-01-A</v>
       </c>
       <c r="B3" s="2" t="str">
-        <v>Gas insulated switchgear side B</v>
+        <v>Gas insulated switchgear side A</v>
       </c>
       <c r="C3" s="2" t="str">
         <v>B14</v>
@@ -491,10 +491,10 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="str">
-        <v>B14-XFM-6041</v>
+        <v>GIS-01-B</v>
       </c>
       <c r="B4" s="2" t="str">
-        <v>Distribution transformer</v>
+        <v>Gas insulated switchgear side B</v>
       </c>
       <c r="C4" s="2" t="str">
         <v>B14</v>
@@ -503,10 +503,10 @@
         <v>Electrical</v>
       </c>
       <c r="E4" s="2" t="str">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="F4" s="2" t="str">
-        <v>Normal Power</v>
+        <v>Medium Voltage</v>
       </c>
       <c r="G4" s="2" t="str">
         <v/>
@@ -517,10 +517,10 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="str">
-        <v>B14-LVS-6041</v>
+        <v>B14-XFM-6041</v>
       </c>
       <c r="B5" s="2" t="str">
-        <v>LV switchboard</v>
+        <v>Distribution transformer</v>
       </c>
       <c r="C5" s="2" t="str">
         <v>B14</v>
@@ -535,7 +535,7 @@
         <v>Normal Power</v>
       </c>
       <c r="G5" s="2" t="str">
-        <v>B14-PP-9999</v>
+        <v/>
       </c>
       <c r="H5" s="2" t="str">
         <v>New</v>
@@ -543,13 +543,13 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="str">
-        <v>B31-XFM-7777</v>
+        <v>B14-LVS-6041</v>
       </c>
       <c r="B6" s="2" t="str">
-        <v>Remote building transformer</v>
+        <v>LV switchboard</v>
       </c>
       <c r="C6" s="2" t="str">
-        <v>B31</v>
+        <v>B14</v>
       </c>
       <c r="D6" s="2" t="str">
         <v>Electrical</v>
@@ -561,7 +561,7 @@
         <v>Normal Power</v>
       </c>
       <c r="G6" s="2" t="str">
-        <v/>
+        <v>B14-PP-9999</v>
       </c>
       <c r="H6" s="2" t="str">
         <v>New</v>
@@ -569,22 +569,22 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="str">
-        <v>B14-RIO-6500</v>
+        <v>B31-XFM-7777</v>
       </c>
       <c r="B7" s="2" t="str">
-        <v>Remote IO panel</v>
+        <v>Remote building transformer</v>
       </c>
       <c r="C7" s="2" t="str">
-        <v>B14</v>
+        <v>B31</v>
       </c>
       <c r="D7" s="2" t="str">
-        <v>I&amp;C</v>
+        <v>Electrical</v>
       </c>
       <c r="E7" s="2" t="str">
-        <v>650</v>
+        <v>604</v>
       </c>
       <c r="F7" s="2" t="str">
-        <v>FMS Network</v>
+        <v>Normal Power</v>
       </c>
       <c r="G7" s="2" t="str">
         <v/>
@@ -593,9 +593,35 @@
         <v>New</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="2" t="str">
+        <v>B14-RIO-6500</v>
+      </c>
+      <c r="B8" s="2" t="str">
+        <v>Remote IO panel</v>
+      </c>
+      <c r="C8" s="2" t="str">
+        <v>B14</v>
+      </c>
+      <c r="D8" s="2" t="str">
+        <v>I&amp;C</v>
+      </c>
+      <c r="E8" s="2" t="str">
+        <v>650</v>
+      </c>
+      <c r="F8" s="2" t="str">
+        <v>FMS Network</v>
+      </c>
+      <c r="G8" s="2" t="str">
+        <v/>
+      </c>
+      <c r="H8" s="2" t="str">
+        <v>New</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>